<commit_message>
Wall port mapping updates
</commit_message>
<xml_diff>
--- a/HCRO/HCRO-Network-Infrastructure/Network-Wall-Port-Mapping.xlsx
+++ b/HCRO/HCRO-Network-Infrastructure/Network-Wall-Port-Mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/smeyers/Documents/GitHubSETI/Front-Page/HCRO/HCRO-Network-Infrastructure/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5F77D5E-A974-F34A-B54E-4A1314416559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ACA296F-EAC0-0246-949F-92E7B7C107F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16480" yWindow="9020" windowWidth="27640" windowHeight="16940" xr2:uid="{4E213348-FF62-B440-B59C-815E7F096F2E}"/>
+    <workbookView xWindow="30880" yWindow="8960" windowWidth="27640" windowHeight="16940" xr2:uid="{4E213348-FF62-B440-B59C-815E7F096F2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -529,6 +529,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB022DAA-1B20-E745-BC0A-55D8341CF941}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -550,7 +551,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -564,7 +565,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -578,7 +579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -592,7 +593,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -606,7 +607,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -620,7 +621,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -634,7 +635,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -648,7 +649,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -662,7 +663,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -676,7 +677,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -690,7 +691,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -704,7 +705,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -718,7 +719,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -732,7 +733,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -746,7 +747,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -760,7 +761,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -774,7 +775,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -788,7 +789,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -802,7 +803,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>15</v>
       </c>
@@ -816,7 +817,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>15</v>
       </c>
@@ -830,7 +831,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>30</v>
       </c>
@@ -844,7 +845,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -886,7 +887,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -900,7 +901,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -914,7 +915,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>15</v>
       </c>
@@ -928,7 +929,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>15</v>
       </c>
@@ -942,7 +943,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>15</v>
       </c>
@@ -956,7 +957,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>15</v>
       </c>
@@ -970,7 +971,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>12</v>
       </c>
@@ -984,7 +985,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>12</v>
       </c>
@@ -998,7 +999,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>12</v>
       </c>
@@ -1012,7 +1013,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>12</v>
       </c>
@@ -1110,7 +1111,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>18</v>
       </c>
@@ -1124,7 +1125,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>18</v>
       </c>
@@ -1138,7 +1139,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>18</v>
       </c>
@@ -1152,7 +1153,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>18</v>
       </c>
@@ -1166,7 +1167,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>18</v>
       </c>
@@ -1180,7 +1181,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>18</v>
       </c>
@@ -1194,7 +1195,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>23</v>
       </c>
@@ -1208,7 +1209,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>23</v>
       </c>
@@ -1222,7 +1223,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>23</v>
       </c>
@@ -1236,7 +1237,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>23</v>
       </c>
@@ -1250,7 +1251,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>23</v>
       </c>
@@ -1264,7 +1265,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>23</v>
       </c>
@@ -1334,7 +1335,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>18</v>
       </c>
@@ -1348,7 +1349,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>18</v>
       </c>
@@ -1362,7 +1363,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>30</v>
       </c>
@@ -1376,7 +1377,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>30</v>
       </c>
@@ -1390,7 +1391,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>18</v>
       </c>
@@ -1404,7 +1405,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>18</v>
       </c>
@@ -1418,7 +1419,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>18</v>
       </c>
@@ -1432,7 +1433,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>18</v>
       </c>
@@ -1446,7 +1447,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>18</v>
       </c>
@@ -1460,7 +1461,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>18</v>
       </c>
@@ -1474,7 +1475,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>30</v>
       </c>
@@ -1488,7 +1489,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>30</v>
       </c>
@@ -1502,7 +1503,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>4</v>
       </c>
@@ -1516,7 +1517,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>4</v>
       </c>
@@ -1530,7 +1531,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>34</v>
       </c>
@@ -1544,7 +1545,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>34</v>
       </c>
@@ -1560,6 +1561,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D73" xr:uid="{BB022DAA-1B20-E745-BC0A-55D8341CF941}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Admin/Student/Sean's Office"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A18:D71">
       <sortCondition ref="D1:D71"/>
     </sortState>

</xml_diff>